<commit_message>
Ajout d'un critere pass fail sur la distance cube-miroir
</commit_message>
<xml_diff>
--- a/assets/config_app.xlsx
+++ b/assets/config_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joudin\Documents\Produits\Lidar\MAPPAL3D\2-OUTILLAGE\SOFTS\Harmonisation\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B9BE24-547B-4E59-A7AC-AFAF046F03CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E103D2CC-293A-4FD7-A79C-083B909B8C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D71F4690-DA34-4EEB-88FE-26DBD695951A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>--</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>SERIAL_NUMBER</t>
+  </si>
+  <si>
+    <t>EUCLIDIAN_DISTANCE_CUBE_MIROR_THRESHOLD_IN_PX</t>
   </si>
 </sst>
 </file>
@@ -426,16 +429,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A6CDD0-E2E0-4645-9A4A-89F3A2106EBA}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="47.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -443,13 +447,16 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,13 +464,16 @@
         <v>0</v>
       </c>
       <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -471,52 +481,52 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>401</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>403</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>404</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>405</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>406</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>407</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>408</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>409</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>410</v>
       </c>

</xml_diff>

<commit_message>
Ajout seuil pass fail centrage emission
</commit_message>
<xml_diff>
--- a/assets/config_app.xlsx
+++ b/assets/config_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joudin\Documents\Produits\Lidar\MAPPAL3D\2-OUTILLAGE\SOFTS\Harmonisation\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E103D2CC-293A-4FD7-A79C-083B909B8C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8CA1071-A38C-4B74-9C02-DBB7176E4C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D71F4690-DA34-4EEB-88FE-26DBD695951A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>--</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>EUCLIDIAN_DISTANCE_CUBE_MIROR_THRESHOLD_IN_PX</t>
+  </si>
+  <si>
+    <t>APD_CENTERS_DISTANCE_THRESHOLD_IN_PX</t>
   </si>
 </sst>
 </file>
@@ -429,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A6CDD0-E2E0-4645-9A4A-89F3A2106EBA}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
@@ -437,9 +440,10 @@
     <col min="3" max="3" width="48.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="47.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -455,8 +459,11 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,8 +479,11 @@
       <c r="E2">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -481,52 +491,52 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>401</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>403</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>404</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>405</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>406</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>407</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>408</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>409</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>410</v>
       </c>

</xml_diff>

<commit_message>
Ajout des numeros RMA à traiter
</commit_message>
<xml_diff>
--- a/assets/config_app.xlsx
+++ b/assets/config_app.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joudin\Documents\Produits\Lidar\MAPPAL3D\2-OUTILLAGE\SOFTS\Harmonisation\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8CA1071-A38C-4B74-9C02-DBB7176E4C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FF2E8A-DDDC-4316-A0AD-6B68F6C58E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D71F4690-DA34-4EEB-88FE-26DBD695951A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D71F4690-DA34-4EEB-88FE-26DBD695951A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>--</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>APD_CENTERS_DISTANCE_THRESHOLD_IN_PX</t>
+  </si>
+  <si>
+    <t>RMA_19</t>
+  </si>
+  <si>
+    <t>RMA_20</t>
   </si>
 </sst>
 </file>
@@ -432,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A6CDD0-E2E0-4645-9A4A-89F3A2106EBA}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
@@ -487,57 +493,67 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>400</v>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>401</v>
+      <c r="B4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B13">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B15">
         <v>410</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Passage en camera reelle. Ajustement des SN
</commit_message>
<xml_diff>
--- a/assets/config_app.xlsx
+++ b/assets/config_app.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joudin\Documents\Produits\Lidar\MAPPAL3D\2-OUTILLAGE\SOFTS\Harmonisation\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FF2E8A-DDDC-4316-A0AD-6B68F6C58E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1687BF22-605D-4E07-A3BC-DB953B47B26D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D71F4690-DA34-4EEB-88FE-26DBD695951A}"/>
   </bookViews>
@@ -62,10 +62,10 @@
     <t>APD_CENTERS_DISTANCE_THRESHOLD_IN_PX</t>
   </si>
   <si>
-    <t>RMA_19</t>
-  </si>
-  <si>
-    <t>RMA_20</t>
+    <t>L-0426-0388</t>
+  </si>
+  <si>
+    <t>L-0426-0389</t>
   </si>
 </sst>
 </file>
@@ -438,11 +438,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A6CDD0-E2E0-4645-9A4A-89F3A2106EBA}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="47.21875" bestFit="1" customWidth="1"/>
@@ -480,7 +480,7 @@
         <v>10</v>
       </c>
       <c r="D2">
-        <v>0.55000000000000004</v>
+        <v>0.5</v>
       </c>
       <c r="E2">
         <v>10</v>
@@ -500,61 +500,6 @@
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15">
-        <v>410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>